<commit_message>
docs(matriz): registrar SHA nuevos de I-001 y de las fases R/D/T/M
Actualiza la matriz y el README con los commits que documentan el código y la documentación pendientes en GitHub.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/documents/matriz_doble_entrada/MATRIZ-DOBLE-ENTRADA-V3-SIGEMAD-MPA.xlsx
+++ b/documents/matriz_doble_entrada/MATRIZ-DOBLE-ENTRADA-V3-SIGEMAD-MPA.xlsx
@@ -877,7 +877,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>7a1c402</t>
+          <t>56e7134</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="Z2" s="22" t="inlineStr">
         <is>
-          <t>Commit 5ce7575 (migración V2 JWT). También AuthMiddleware.php, Jwt.php y AuthContext.jsx. Historial Git agregado (no un commit por prompt). Sin prueba unitaria de login.</t>
+          <t>Origen JWT: 5ce7575. Claim nombre_completo en login: 4e08b9e [I-001]. También AuthMiddleware.php, Jwt.php y AuthContext.jsx. Sin prueba unitaria de login.</t>
         </is>
       </c>
     </row>
@@ -1321,12 +1321,12 @@
       </c>
       <c r="U3" s="27" t="inlineStr">
         <is>
-          <t>https://github.com/AxlTech25/Gestion-MPA/blob/9950f99/src/features/configuracion/components/ConfiguracionPage.jsx</t>
+          <t>https://github.com/AxlTech25/Gestion-MPA/blob/4e08b9e/src/features/configuracion/components/ConfiguracionPage.jsx</t>
         </is>
       </c>
       <c r="V3" s="27" t="inlineStr">
         <is>
-          <t>9950f99</t>
+          <t>4e08b9e</t>
         </is>
       </c>
       <c r="W3" s="26" t="inlineStr">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="Z3" s="26" t="inlineStr">
         <is>
-          <t>Commit 9950f99 (estructura inicial; incremento 5 v0.5.0 via en ese lote). API: AreaController.php y UsuarioController.php.</t>
+          <t>SHA vigente: 4e08b9e [I-001] (nombre completo y UI de usuarios). Origen del módulo: 9950f99. API: AreaController.php y UsuarioController.php.</t>
         </is>
       </c>
     </row>
@@ -1451,12 +1451,12 @@
       </c>
       <c r="U4" s="25" t="inlineStr">
         <is>
-          <t>https://github.com/AxlTech25/Gestion-MPA/blob/9950f99/backend/api/v2/controllers/EquipoController.php</t>
+          <t>https://github.com/AxlTech25/Gestion-MPA/blob/f086a63/backend/api/v2/controllers/EquipoController.php</t>
         </is>
       </c>
       <c r="V4" s="25" t="inlineStr">
         <is>
-          <t>9950f99</t>
+          <t>f086a63</t>
         </is>
       </c>
       <c r="W4" s="22" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="Z4" s="22" t="inlineStr">
         <is>
-          <t>Commit 9950f99 (origen del CRUD). Evoluciones posteriores en 06d75b1 y 1c63dbe. Test unitario solo de tipo de equipo (Vitest).</t>
+          <t>SHA vigente: f086a63 [I-001] (evaluación, PDF y esquema). Origen del CRUD: 9950f99. Test unitario solo de tipo de equipo (Vitest).</t>
         </is>
       </c>
     </row>
@@ -1581,12 +1581,12 @@
       </c>
       <c r="U5" s="27" t="inlineStr">
         <is>
-          <t>https://github.com/AxlTech25/Gestion-MPA/blob/9950f99/backend/api/v2/controllers/FichaTecnicaController.php</t>
+          <t>https://github.com/AxlTech25/Gestion-MPA/blob/f086a63/backend/api/v2/controllers/FichaTecnicaController.php</t>
         </is>
       </c>
       <c r="V5" s="27" t="inlineStr">
         <is>
-          <t>9950f99</t>
+          <t>f086a63</t>
         </is>
       </c>
       <c r="W5" s="26" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="Z5" s="26" t="inlineStr">
         <is>
-          <t>Commit 9950f99 (origen). UI: FichaTecnicaPage.jsx y FichaTecnicaPanel.jsx. Bloque predictivo en 8b20337 (v0.9.0).</t>
+          <t>SHA vigente: f086a63 [I-001] (FichaTecnicaController y panel). Origen: 9950f99. Bloque predictivo: 8b20337 (v0.9.0).</t>
         </is>
       </c>
     </row>
@@ -2101,12 +2101,12 @@
       </c>
       <c r="U9" s="27" t="inlineStr">
         <is>
-          <t>https://github.com/AxlTech25/Gestion-MPA/blob/5ce7575/backend/api/v2/controllers/ReporteController.php</t>
+          <t>https://github.com/AxlTech25/Gestion-MPA/blob/f086a63/backend/api/v2/controllers/ReporteController.php</t>
         </is>
       </c>
       <c r="V9" s="27" t="inlineStr">
         <is>
-          <t>5ce7575</t>
+          <t>f086a63</t>
         </is>
       </c>
       <c r="W9" s="26" t="inlineStr">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="Z9" s="26" t="inlineStr">
         <is>
-          <t>Commit 5ce7575 (descarga PDF con JWT). Origen del controlador: 9950f99. Sin prueba unitaria del PDF.</t>
+          <t>SHA vigente: f086a63 [I-001] (ReporteController y downloadPdf). JWT en blob: 5ce7575. Origen: 9950f99.</t>
         </is>
       </c>
     </row>
@@ -2300,7 +2300,7 @@
       </c>
       <c r="K2" s="25" t="inlineStr">
         <is>
-          <t>prompts/03_implementacion/I-001_api_auth_inventario_v1.md · Código: 9950f99 (origen), 5ce7575 (JWT/dashboard). Ver columna Commit de F-001 a F-006 y F-008.</t>
+          <t>prompts/03_implementacion/I-001_api_auth_inventario_v1.md · Vigente: f086a63 (inventario/ficha/PDF), 4e08b9e (configuración). Origen: 9950f99, JWT: 5ce7575.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(matriz): publicar prompts detallados por función F-001 a F-008
Deja en main la hoja Jiang (prompt exacto, técnica, iteraciones y commit) y los I-00N vigentes que el Excel enlaza.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/documents/matriz_doble_entrada/MATRIZ-DOBLE-ENTRADA-V3-SIGEMAD-MPA.xlsx
+++ b/documents/matriz_doble_entrada/MATRIZ-DOBLE-ENTRADA-V3-SIGEMAD-MPA.xlsx
@@ -685,7 +685,7 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Aporta el modelo de versionado y gestión de calidad de prompts (control de iteraciones, criterio de aceptación). Se refleja en 'ID Prompt', 'Versión del prompt', 'N.º de iteraciones' y 'Criterio de aceptación'. En Sigemad los IDs siguen el repositorio prompts/: I-001 (API V2 e inventario) e I-002 (microservicio ML).</t>
+          <t>Aporta el modelo de versionado y gestión de calidad de prompts (control de iteraciones, criterio de aceptación). Se refleja en 'ID Prompt', 'Versión del prompt', 'N.º de iteraciones' y 'Criterio de aceptación'. En Sigemad los IDs vigentes son I-002…I-009 (una fila por función F-001…F-008 en Prompts Detallados).</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>Al mantener el sistema: 1) registra o reutiliza un prompt en prompts/; 2) implementa el cambio; 3) haz commit con el ID del prompt en el mensaje, p. ej. feat(inventario): validar código [I-001]; 4) actualiza SHA, Link GitHub y N.º de iteraciones en esta matriz.</t>
+          <t>Al mantener el sistema: 1) registra o reutiliza un prompt en prompts/; 2) implementa el cambio; 3) haz commit con el ID del prompt en el mensaje, p. ej. feat(inventario): validar código [I-002]; 4) actualiza SHA, Link GitHub y N.º de iteraciones en esta matriz.</t>
         </is>
       </c>
     </row>
@@ -804,7 +804,7 @@
     <row r="20" ht="42" customHeight="1" s="14">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>Explica que las 5 columnas DevOps operan bajo Amaro et al. (2025); las de prompt versionado bajo Jiang et al. (2025); y que la trazabilidad de mantenimiento es prompt → commit GitHub → archivo (síntesis original del caso Sigemad). Limitación: el historial Git anterior a esta matriz es agregado (pocos commits grandes), no un SHA por cada prompt; I-001 e I-002 se documentaron de forma retrospectiva (metodologia.md §7). A partir de este registro, cada cambio asistido por IA debe dejar SHA propio.</t>
+          <t>Explica que las 5 columnas DevOps operan bajo Amaro et al. (2025); las de prompt versionado bajo Jiang et al. (2025); y que la trazabilidad de mantenimiento es prompt → commit GitHub → archivo (síntesis original del caso Sigemad). Limitación: el historial Git anterior a esta matriz es agregado (pocos commits grandes), no un SHA por cada prompt; los I-00N se documentaron de forma retrospectiva (metodologia.md). A partir de este registro, cada cambio asistido por IA debe dejar SHA propio.</t>
         </is>
       </c>
     </row>
@@ -913,7 +913,7 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>tipo(modulo): mensaje [I-001]  — ejemplo: feat(inventario): filtro por área [I-001]</t>
+          <t>tipo(modulo): mensaje [I-002]  — ejemplo: feat(inventario): filtro por área [I-002]</t>
         </is>
       </c>
     </row>
@@ -1148,12 +1148,12 @@
       </c>
       <c r="L2" s="25" t="inlineStr">
         <is>
-          <t>I-001</t>
+          <t>I-006</t>
         </is>
       </c>
       <c r="M2" s="22" t="inlineStr">
         <is>
-          <t>Zero-shot</t>
+          <t>CoT guiado</t>
         </is>
       </c>
       <c r="N2" s="22" t="inlineStr">
@@ -1216,7 +1216,7 @@
       </c>
       <c r="Z2" s="22" t="inlineStr">
         <is>
-          <t>Origen JWT: 5ce7575. Claim nombre_completo en login: 4e08b9e [I-001]. También AuthMiddleware.php, Jwt.php y AuthContext.jsx. Sin prueba unitaria de login.</t>
+          <t>Origen JWT: 5ce7575 [I-006]. RBAC en servidor: I-009. También AuthMiddleware.php, Jwt.php y AuthContext.jsx.</t>
         </is>
       </c>
     </row>
@@ -1278,12 +1278,12 @@
       </c>
       <c r="L3" s="27" t="inlineStr">
         <is>
-          <t>I-001</t>
+          <t>I-005</t>
         </is>
       </c>
       <c r="M3" s="26" t="inlineStr">
         <is>
-          <t>Zero-shot</t>
+          <t>Few-shot</t>
         </is>
       </c>
       <c r="N3" s="26" t="inlineStr">
@@ -1292,7 +1292,7 @@
         </is>
       </c>
       <c r="O3" s="26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P3" s="26" t="inlineStr">
         <is>
@@ -1346,7 +1346,7 @@
       </c>
       <c r="Z3" s="26" t="inlineStr">
         <is>
-          <t>SHA vigente: 4e08b9e [I-001] (nombre completo y UI de usuarios). Origen del módulo: 9950f99. API: AreaController.php y UsuarioController.php.</t>
+          <t>SHA vigente: 4e08b9e [I-005]. requireRole Administrador: I-009. API: AreaController.php y UsuarioController.php.</t>
         </is>
       </c>
     </row>
@@ -1408,12 +1408,12 @@
       </c>
       <c r="L4" s="25" t="inlineStr">
         <is>
-          <t>I-001</t>
+          <t>I-002</t>
         </is>
       </c>
       <c r="M4" s="22" t="inlineStr">
         <is>
-          <t>Zero-shot</t>
+          <t>Few-shot</t>
         </is>
       </c>
       <c r="N4" s="22" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="Z4" s="22" t="inlineStr">
         <is>
-          <t>SHA vigente: f086a63 [I-001] (evaluación, PDF y esquema). Origen del CRUD: 9950f99. Test unitario solo de tipo de equipo (Vitest).</t>
+          <t>SHA vigente: f086a63 [I-002]. Telemetría: I-008. Plantilla Excel: I-009. Test unitario de tipo de equipo (Vitest).</t>
         </is>
       </c>
     </row>
@@ -1538,12 +1538,12 @@
       </c>
       <c r="L5" s="27" t="inlineStr">
         <is>
-          <t>I-001</t>
+          <t>I-003</t>
         </is>
       </c>
       <c r="M5" s="26" t="inlineStr">
         <is>
-          <t>Zero-shot</t>
+          <t>Few-shot</t>
         </is>
       </c>
       <c r="N5" s="26" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="Z5" s="26" t="inlineStr">
         <is>
-          <t>SHA vigente: f086a63 [I-001] (FichaTecnicaController y panel). Origen: 9950f99. Bloque predictivo: 8b20337 (v0.9.0).</t>
+          <t>SHA vigente: f086a63 [I-003]. Bloque predictivo en ficha: 8b20337 [I-008].</t>
         </is>
       </c>
     </row>
@@ -1668,12 +1668,12 @@
       </c>
       <c r="L6" s="25" t="inlineStr">
         <is>
-          <t>I-001</t>
+          <t>I-003</t>
         </is>
       </c>
       <c r="M6" s="22" t="inlineStr">
         <is>
-          <t>Zero-shot</t>
+          <t>Few-shot</t>
         </is>
       </c>
       <c r="N6" s="22" t="inlineStr">
@@ -1736,7 +1736,7 @@
       </c>
       <c r="Z6" s="22" t="inlineStr">
         <is>
-          <t>Commit 8b20337 (v0.9.0 telemetría y correctivo estructurado). Origen del módulo: 9950f99. PHPUnit: sync de telemetría.</t>
+          <t>SHA de timeline/categoría: 8b20337 [I-003]. Sync de telemetría: I-008. PHPUnit: sync de telemetría.</t>
         </is>
       </c>
     </row>
@@ -1798,12 +1798,12 @@
       </c>
       <c r="L7" s="27" t="inlineStr">
         <is>
-          <t>I-001</t>
+          <t>I-006</t>
         </is>
       </c>
       <c r="M7" s="26" t="inlineStr">
         <is>
-          <t>Zero-shot</t>
+          <t>CoT guiado</t>
         </is>
       </c>
       <c r="N7" s="26" t="inlineStr">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="Z7" s="26" t="inlineStr">
         <is>
-          <t>Commit 5ce7575 (dashboard de métricas + JWT). Alertas ML y consulta: 8b20337. PHPUnit cubre filtros de consulta. Monitoring de software = No.</t>
+          <t>Commit 5ce7575 [I-006] (dashboard de métricas + JWT). Alertas ML: I-007. Consulta tipo_otro: I-008.</t>
         </is>
       </c>
     </row>
@@ -1928,12 +1928,12 @@
       </c>
       <c r="L8" s="25" t="inlineStr">
         <is>
-          <t>I-002</t>
+          <t>I-007</t>
         </is>
       </c>
       <c r="M8" s="22" t="inlineStr">
         <is>
-          <t>Zero-shot</t>
+          <t>CoT guiado</t>
         </is>
       </c>
       <c r="N8" s="22" t="inlineStr">
@@ -1942,7 +1942,7 @@
         </is>
       </c>
       <c r="O8" s="22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P8" s="22" t="inlineStr">
         <is>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="Z8" s="22" t="inlineStr">
         <is>
-          <t>Commit e9a0965 (FastAPI). Proxy PHP y cierre v0.9.0: 06d75b1 / 8b20337. pytest: test_features.py y test_ml_schemas.py. ML opcional.</t>
+          <t>Commit e9a0965 [I-007] (FastAPI). Telemetría/ficha predictiva: I-008. pytest: test_features.py y test_ml_schemas.py.</t>
         </is>
       </c>
     </row>
@@ -2058,12 +2058,12 @@
       </c>
       <c r="L9" s="27" t="inlineStr">
         <is>
-          <t>I-001</t>
+          <t>I-004</t>
         </is>
       </c>
       <c r="M9" s="26" t="inlineStr">
         <is>
-          <t>Zero-shot</t>
+          <t>Zero-shot + few-shot</t>
         </is>
       </c>
       <c r="N9" s="26" t="inlineStr">
@@ -2072,7 +2072,7 @@
         </is>
       </c>
       <c r="O9" s="26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P9" s="26" t="inlineStr">
         <is>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="Z9" s="26" t="inlineStr">
         <is>
-          <t>SHA vigente: f086a63 [I-001] (ReporteController y downloadPdf). JWT en blob: 5ce7575. Origen: 9950f99.</t>
+          <t>SHA vigente: f086a63 [I-004]. Descarga con JWT (blob): 5ce7575 [I-006].</t>
         </is>
       </c>
     </row>
@@ -2178,18 +2178,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
-    <col width="10" customWidth="1" style="14" min="1" max="1"/>
-    <col width="14" customWidth="1" style="14" min="2" max="2"/>
-    <col width="60" customWidth="1" style="14" min="3" max="3"/>
-    <col width="16" customWidth="1" style="14" min="4" max="4"/>
+    <col width="12" customWidth="1" style="14" min="1" max="1"/>
+    <col width="28" customWidth="1" style="14" min="2" max="2"/>
+    <col width="72" customWidth="1" style="14" min="3" max="3"/>
+    <col width="18" customWidth="1" style="14" min="4" max="4"/>
     <col width="12" customWidth="1" style="14" min="5" max="6"/>
     <col width="28" customWidth="1" style="14" min="7" max="7"/>
     <col width="12" customWidth="1" style="14" min="8" max="9"/>
     <col width="24" customWidth="1" style="14" min="10" max="10"/>
-    <col width="14" customWidth="1" style="14" min="11" max="11"/>
+    <col width="16" customWidth="1" style="14" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="14">
@@ -2252,22 +2252,22 @@
     <row r="2" ht="90" customHeight="1" s="14">
       <c r="A2" s="25" t="inlineStr">
         <is>
-          <t>I-001</t>
+          <t>I-006</t>
         </is>
       </c>
       <c r="B2" s="22" t="inlineStr">
         <is>
-          <t>F-001 a F-006, F-008</t>
+          <t>F-001</t>
         </is>
       </c>
       <c r="C2" s="22" t="inlineStr">
         <is>
-          <t>Actúa como un desarrollador senior PHP/React. Contexto: API en backend/api/v2, frontend organizado por features, JWT y RBAC (Administrador, Técnico, Practicante). Implementa autenticación, CRUD de equipos, fichas técnicas, mantenimientos, áreas, usuarios, dashboard y reportes PDF. Restricciones: respuestas JSON estándar {success, data, message}; middleware JWT en todas las rutas salvo /auth; código patrimonial de 12 dígitos. No inventar integraciones SIGA/SIAF ni portal ciudadano.</t>
+          <t>Actúa como desarrollador senior PHP (firebase/php-jwt) y React (AuthContext, Axios). Contexto: API v2 y módulos INV/MNT/CFG sin JWT obligatorio; ADR-001 exige Bearer salvo /auth. Objetivo: login, sesión persistente y protección de /v2/* y de la API. Tarea: POST /auth/login → JWT; AuthMiddleware::requireAuth excepto /auth; Login.jsx, AuthContext, PrivateRoute; interceptor Axios; 401 → login; Navbar con Salir. Restricciones: secret solo en config no versionada; no revelar si el usuario existe; no FastAPI. Criterios: login correcto → /v2/dashboard; F5 mantiene sesión; sin token API 401.</t>
         </is>
       </c>
       <c r="D2" s="22" t="inlineStr">
         <is>
-          <t>Zero-shot</t>
+          <t>CoT guiado</t>
         </is>
       </c>
       <c r="E2" s="22" t="inlineStr">
@@ -2280,7 +2280,7 @@
       </c>
       <c r="G2" s="22" t="inlineStr">
         <is>
-          <t>Registro retrospectivo en prompts/; aprobado en primera versión documentada (incrementos 1–6, v0.1.0–0.6.0).</t>
+          <t>N/A — aprobado en primera versión documentada. El endurecimiento de roles es I-009.</t>
         </is>
       </c>
       <c r="H2" s="22" t="inlineStr">
@@ -2295,84 +2295,532 @@
       </c>
       <c r="J2" s="22" t="inlineStr">
         <is>
-          <t>API V2 + features React de auth, configuración, inventario, ficha, mantenimiento, dashboard y reportes</t>
+          <t>Login JWT funcional (AuthContext, PrivateRoute, middleware)</t>
         </is>
       </c>
       <c r="K2" s="25" t="inlineStr">
         <is>
-          <t>prompts/03_implementacion/I-001_api_auth_inventario_v1.md · Vigente: f086a63 (inventario/ficha/PDF), 4e08b9e (configuración). Origen: 9950f99, JWT: 5ce7575.</t>
+          <t>5ce7575</t>
         </is>
       </c>
     </row>
     <row r="3" ht="90" customHeight="1" s="14">
       <c r="A3" s="27" t="inlineStr">
         <is>
+          <t>I-005</t>
+        </is>
+      </c>
+      <c r="B3" s="26" t="inlineStr">
+        <is>
+          <t>F-002</t>
+        </is>
+      </c>
+      <c r="C3" s="26" t="inlineStr">
+        <is>
+          <t>Actúa como desarrollador senior PHP/React. Contexto: áreas y responsables no deben estar hardcodeados en EquipoForm; tablas v2_areas y v2_usuarios existen; ruta /v2/configuracion; roles Administrador, Tecnico, Practicante. Objetivo: CRUD de áreas y alta/listado de personal. Tarea: modelos PDO; password_hash BCRYPT; rutas /areas y /usuarios; ConfiguracionPage (pestañas); EquipoForm consume áreas desde API. Restricciones: no MD5; no requireRole en este incremento (deuda → I-009). Criterios: crear un área y verla en EquipoForm; usuario con hash en BD.</t>
+        </is>
+      </c>
+      <c r="D3" s="26" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="E3" s="26" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F3" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="26" t="inlineStr">
+        <is>
+          <t>La API de usuarios quedó solo autenticada. I-009 añade requireRole Administrador.</t>
+        </is>
+      </c>
+      <c r="H3" s="26" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I3" s="26" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="J3" s="26" t="inlineStr">
+        <is>
+          <t>Áreas y personal funcionales; EquipoForm dinámico</t>
+        </is>
+      </c>
+      <c r="K3" s="27" t="inlineStr">
+        <is>
+          <t>4e08b9e</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="90" customHeight="1" s="14">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
           <t>I-002</t>
         </is>
       </c>
-      <c r="B3" s="26" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
+        <is>
+          <t>F-003</t>
+        </is>
+      </c>
+      <c r="C4" s="22" t="inlineStr">
+        <is>
+          <t>Actúa como desarrollador senior PHP/React sobre el esqueleto I-001. Contexto: v2_equipos ya existe; CRUD mínimo ML-ready (ram_gb, almacenamiento_gb, fechas); código patrimonial de 12 dígitos; tabla + modal Tailwind. Objetivo: listado y alta vía /api/v2/equipos y src/features/inventario, sin fichas ni PDF. Tarea: Equipo.php (getAll, create); EquipoController JSON {success, data, message}; InventarioPage y EquipoForm. Restricciones: 12 dígitos únicos; no texto “8 GB”; no FastAPI. Criterios: POST persiste y GET lista; el form rechaza código ≠ 12.</t>
+        </is>
+      </c>
+      <c r="D4" s="22" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="E4" s="22" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F4" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="22" t="inlineStr">
+        <is>
+          <t>N/A — no confundir con I-002-ML histórico (ahora I-007).</t>
+        </is>
+      </c>
+      <c r="H4" s="22" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I4" s="22" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="J4" s="22" t="inlineStr">
+        <is>
+          <t>CRUD de equipos con código de 12 dígitos y RAM numérica</t>
+        </is>
+      </c>
+      <c r="K4" s="25" t="inlineStr">
+        <is>
+          <t>f086a63</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="90" customHeight="1" s="14">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>I-003</t>
+        </is>
+      </c>
+      <c r="B5" s="26" t="inlineStr">
+        <is>
+          <t>F-004</t>
+        </is>
+      </c>
+      <c r="C5" s="26" t="inlineStr">
+        <is>
+          <t>Actúa como desarrollador senior PHP/React; replica el patrón I-002. Contexto: equipos ya se listan; hace falta consultar/editar ficha técnica del equipo. Tarea: modelo/controlador/ruta de fichas; GET por id y por código patrimonial; acceso desde inventario (modal o /v2/ficha-tecnica). Restricciones: no PDF (I-004); no bloque ML (I-008). Criterios: GET ficha existente o vacío controlado (no 500).</t>
+        </is>
+      </c>
+      <c r="D5" s="26" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="E5" s="26" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F5" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="26" t="inlineStr">
+        <is>
+          <t>N/A — evaluación predictiva en ficha es I-008.</t>
+        </is>
+      </c>
+      <c r="H5" s="26" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I5" s="26" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="J5" s="26" t="inlineStr">
+        <is>
+          <t>API y UI de ficha técnica por id o código</t>
+        </is>
+      </c>
+      <c r="K5" s="27" t="inlineStr">
+        <is>
+          <t>f086a63</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="90" customHeight="1" s="14">
+      <c r="A6" s="25" t="inlineStr">
+        <is>
+          <t>I-003</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>F-005</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>Actúa como desarrollador senior PHP/React; patrón I-002. Contexto: historial de intervenciones con categoria_falla_id del catálogo v2_categorias_falla; no texto libre como verdad de la falla. Objetivo: registrar y listar mantenimientos. Tarea: Mantenimiento.php getAll (JOIN categoría y técnico) y create; timeline + modal; select de categoría. Restricciones: categoría obligatoria en correctivo; no telemetría (I-008); no ML (I-007). Criterios: POST liga equipo_id; timeline muestra fecha, tipo y categoría nombrada.</t>
+        </is>
+      </c>
+      <c r="D6" s="22" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="E6" s="22" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="22" t="inlineStr">
+        <is>
+          <t>N/A — sync de telemetría es I-008.</t>
+        </is>
+      </c>
+      <c r="H6" s="22" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I6" s="22" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="J6" s="22" t="inlineStr">
+        <is>
+          <t>Timeline y alta estructurada de mantenimientos</t>
+        </is>
+      </c>
+      <c r="K6" s="25" t="inlineStr">
+        <is>
+          <t>8b20337</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="90" customHeight="1" s="14">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>I-006</t>
+        </is>
+      </c>
+      <c r="B7" s="26" t="inlineStr">
+        <is>
+          <t>F-006</t>
+        </is>
+      </c>
+      <c r="C7" s="26" t="inlineStr">
+        <is>
+          <t>Actúa como desarrollador senior PHP/React (mismo incremento 0.6.0 que F-001). Objetivo: métricas operativas en GET /api/v2/dashboard y UI DashboardPage (conteos, no ML). Tarea: DashboardController + DashboardPage; no badges de riesgo (I-007); no panel de consulta por etiquetas (I-008). Restricciones: no llamar a :8000. Criterios: dashboard muestra conteos persistidos tras login.</t>
+        </is>
+      </c>
+      <c r="D7" s="26" t="inlineStr">
+        <is>
+          <t>CoT guiado</t>
+        </is>
+      </c>
+      <c r="E7" s="26" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F7" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="26" t="inlineStr">
+        <is>
+          <t>N/A — consulta tipo_otro es I-008; alertas ML son I-007.</t>
+        </is>
+      </c>
+      <c r="H7" s="26" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I7" s="26" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="J7" s="26" t="inlineStr">
+        <is>
+          <t>Dashboard de métricas operativas funcional</t>
+        </is>
+      </c>
+      <c r="K7" s="27" t="inlineStr">
+        <is>
+          <t>5ce7575</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="90" customHeight="1" s="14">
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>I-007</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>F-007</t>
         </is>
       </c>
-      <c r="C3" s="26" t="inlineStr">
-        <is>
-          <t>Actúa como ingeniero ML y backend. Contexto: dataset estructurado desde inventario y mantenimientos. Modelo de riesgo por equipo (Random Forest) y sugerencia de categoría de falla. Implementa microservicio FastAPI (entrenamiento e inferencia), tabla v2_predicciones_ml, proxy PHP autenticado /api/v2/ml/*, badges de riesgo en inventario y alertas en dashboard. Restricciones: PHP es el único cliente del puerto 8000; si FastAPI no responde, el resto del sistema continúa (degradación controlada).</t>
-        </is>
-      </c>
-      <c r="D3" s="26" t="inlineStr">
-        <is>
-          <t>Zero-shot</t>
-        </is>
-      </c>
-      <c r="E3" s="26" t="inlineStr">
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>Actúa como ingeniero de ML aplicado y backend PHP. Contexto: datos estructurados (I-002, I-003); JWT (I-006); FastAPI en :8000; PHP único cliente; Hostinger sin Python. Objetivo: riesgo por equipo, sugerencia de categoría, proxy JWT y UI degradable. Tarea: dataset sintético ~200; Random Forest; /health, /predict/riesgo, batch, /predict/categoria, /train; tabla v2_predicciones_ml; proxy /api/v2/ml/*; badges. Restricciones: batch JSON {} no []; si FastAPI cae, inventario y login siguen. Criterios: /health OK; 401 sin token; UI sin crash con uvicorn down.</t>
+        </is>
+      </c>
+      <c r="D8" s="22" t="inlineStr">
+        <is>
+          <t>CoT guiado</t>
+        </is>
+      </c>
+      <c r="E8" s="22" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="F3" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="26" t="inlineStr">
-        <is>
-          <t>Registro retrospectivo en prompts/; aprobado en incrementos 6–7 (v0.7.0–0.9.0).</t>
-        </is>
-      </c>
-      <c r="H3" s="26" t="inlineStr">
+      <c r="F8" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="22" t="inlineStr">
+        <is>
+          <t>Batch enviaba []; curl devolvía HTTP 503 con cuerpo OK.</t>
+        </is>
+      </c>
+      <c r="H8" s="22" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="I3" s="26" t="inlineStr">
+      <c r="I8" s="22" t="inlineStr">
         <is>
           <t>Aprobado</t>
         </is>
       </c>
-      <c r="J3" s="26" t="inlineStr">
-        <is>
-          <t>FastAPI + proxy PHP + UI de riesgo y ficha predictiva; pytest de features y schemas</t>
-        </is>
-      </c>
-      <c r="K3" s="27" t="inlineStr">
-        <is>
-          <t>prompts/03_implementacion/I-002_microservicio_ml_v1.md · Código: e9a0965 (FastAPI), 8b20337 (cierre v0.9.0). Ver F-007.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="101.5" customHeight="1" s="14"/>
-    <row r="5" ht="101.5" customHeight="1" s="14"/>
-    <row r="6" ht="101.5" customHeight="1" s="14"/>
-    <row r="7" ht="101.5" customHeight="1" s="14"/>
-    <row r="8" ht="116" customHeight="1" s="14"/>
-    <row r="9" ht="116" customHeight="1" s="14"/>
-    <row r="10" ht="101.5" customHeight="1" s="14"/>
-    <row r="11" ht="116" customHeight="1" s="14"/>
+      <c r="J8" s="22" t="inlineStr">
+        <is>
+          <t>FastAPI + proxy PHP + badges; degradación controlada</t>
+        </is>
+      </c>
+      <c r="K8" s="25" t="inlineStr">
+        <is>
+          <t>e9a0965</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="90" customHeight="1" s="14">
+      <c r="A9" s="27" t="inlineStr">
+        <is>
+          <t>I-004</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>F-008</t>
+        </is>
+      </c>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>Actúa como desarrollador senior PHP (dompdf) y React. Contexto: inventario y ficha ya existen. Objetivo: GET /api/v2/reportes/equipo/{id} genera PDF; InventarioPage filtra en cliente y ofrece descargar ficha. Tarea: Composer dompdf; ReporteController HTML→PDF; botón en la fila. Restricciones: PDF binario, no base64; no reportes de mantenimiento en este incremento. Criterios: PDF muestra código patrimonial; filtro de texto reduce filas.</t>
+        </is>
+      </c>
+      <c r="D9" s="26" t="inlineStr">
+        <is>
+          <t>Zero-shot + few-shot</t>
+        </is>
+      </c>
+      <c r="E9" s="26" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F9" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="26" t="inlineStr">
+        <is>
+          <t>window.open sin token; I-006 cambia la descarga a blob + Authorization.</t>
+        </is>
+      </c>
+      <c r="H9" s="26" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I9" s="26" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="J9" s="26" t="inlineStr">
+        <is>
+          <t>PDF de ficha y filtros de inventario funcionales</t>
+        </is>
+      </c>
+      <c r="K9" s="27" t="inlineStr">
+        <is>
+          <t>f086a63</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="90" customHeight="1" s="14">
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>I-008</t>
+        </is>
+      </c>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>F-003, F-005, F-006, F-007</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>Actúa como desarrollador PHP/React e ingeniero de datos ML. Contexto: ML 0.7.0 ya opera (I-007). Ampliar v2_equipos y v2_fichas_mantenimiento con telemetría y contexto de intervención; syncTelemetria al registrar mantenimiento; consulta de dashboard; bloque predictivo en ficha. No agente WMI ni DELETE de equipos. Criterios: migrate sobre BD 0.7.0 sin pérdida; POST mantenimiento actualiza snapshot; ficha muestra score si ML está arriba.</t>
+        </is>
+      </c>
+      <c r="D10" s="22" t="inlineStr">
+        <is>
+          <t>CoT guiado</t>
+        </is>
+      </c>
+      <c r="E10" s="22" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F10" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" s="22" t="inlineStr">
+        <is>
+          <t>I-007 no incluía telemetría; D-005 pidió evolución por fases (0.8.0 y 0.9.0).</t>
+        </is>
+      </c>
+      <c r="H10" s="22" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I10" s="22" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="J10" s="22" t="inlineStr">
+        <is>
+          <t>Telemetría, sync, ficha predictiva y consulta de equipos</t>
+        </is>
+      </c>
+      <c r="K10" s="25" t="inlineStr">
+        <is>
+          <t>8b20337</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="90" customHeight="1" s="14">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>I-009</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>F-001, F-002, F-003</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>Actúa como desarrollador senior de API PHP y React. Contexto: 0.9.1; JWT existe; un Técnico puede mutar /usuarios; plantilla Excel desalinea numero_serie/area por falta de color. Objetivo: requireRole Administrador en escritura de usuarios; no autoeliminación ni borrar el último admin; RoleRoute en Configuración; fila ejemplo Excel alineada. Criterios: Técnico en POST /usuarios → 403.</t>
+        </is>
+      </c>
+      <c r="D11" s="26" t="inlineStr">
+        <is>
+          <t>CoT guiado</t>
+        </is>
+      </c>
+      <c r="E11" s="26" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F11" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="26" t="inlineStr">
+        <is>
+          <t>I-005 no puso autorización en servidor (deuda de RBAC).</t>
+        </is>
+      </c>
+      <c r="H11" s="26" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I11" s="26" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="J11" s="26" t="inlineStr">
+        <is>
+          <t>requireRole en /usuarios y plantilla Excel alineada</t>
+        </is>
+      </c>
+      <c r="K11" s="27" t="inlineStr">
+        <is>
+          <t>8b20337</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2604,7 +3052,7 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Identificador del prompt que generó o modificó el módulo (I-001, I-002). En la matriz es un hipervínculo al markdown en GitHub (prompts/).</t>
+          <t>Identificador del prompt vigente (I-002…I-009). Una fila por función F-001…F-008 en Prompts Detallados. Hipervínculo al markdown en GitHub (prompts/).</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">

</xml_diff>

<commit_message>
docs(matriz): anclar F-009 e I-010…I-017 al SHA 3394712 [I-010]
Regenera el Excel de doble entrada ahora que el Incremento 8 está en Git.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/documents/matriz_doble_entrada/MATRIZ-DOBLE-ENTRADA-V3-SIGEMAD-MPA.xlsx
+++ b/documents/matriz_doble_entrada/MATRIZ-DOBLE-ENTRADA-V3-SIGEMAD-MPA.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diccionario de Columnas" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz Consolidada'!$A$1:$Z$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz Consolidada'!$A$1:$Z$10</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -130,12 +130,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -251,16 +251,16 @@
     <xf numFmtId="0" fontId="7" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -685,7 +685,7 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Aporta el modelo de versionado y gestión de calidad de prompts (control de iteraciones, criterio de aceptación). Se refleja en 'ID Prompt', 'Versión del prompt', 'N.º de iteraciones' y 'Criterio de aceptación'. En Sigemad los IDs vigentes son I-002…I-009 (una fila por función F-001…F-008 en Prompts Detallados).</t>
+          <t>Aporta el modelo de versionado y gestión de calidad de prompts (control de iteraciones, criterio de aceptación). Se refleja en 'ID Prompt', 'Versión del prompt', 'N.º de iteraciones' y 'Criterio de aceptación'. En Sigemad los IDs vigentes son I-002…I-017 (una fila por función F-001…F-009 en Prompts Detallados, más refinamientos I-008…I-017).</t>
         </is>
       </c>
     </row>
@@ -717,7 +717,7 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Busca en 'Matriz Consolidada' por 'Feature/Módulo' (auth, inventario, ficha, mantenimiento, dashboard, ml, reportes, configuracion) o 'ID Función' (F-001 a F-008).</t>
+          <t>Busca en 'Matriz Consolidada' por 'Feature/Módulo' (auth, inventario, ficha, mantenimiento, dashboard, ml, reportes, configuracion, cronograma) o 'ID Función' (F-001 a F-009).</t>
         </is>
       </c>
     </row>
@@ -729,7 +729,7 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>Observa las 5 columnas DevOps (Amaro): verde = Sí implementado, amarillo = Parcial, rojo = No implementado. En este caso: Control de Versiones = Sí (Git); CI y CD = No (no hay pipeline GitHub Actions ni despliegue automático; Hostinger es manual); Test Automation = Parcial en inventario, mantenimiento, dashboard y ML; Continuous Monitoring = No.</t>
+          <t>Observa las 5 columnas DevOps (Amaro): verde = Sí implementado, amarillo = Parcial, rojo = No implementado. En este caso: Control de Versiones = Sí (Git); CI y CD = No (no hay pipeline GitHub Actions ni despliegue automático; Hostinger es manual); Test Automation = Parcial en auth, configuración, inventario, mantenimiento, dashboard, ML, reportes (PDF cronograma) y cronograma; Continuous Monitoring = No.</t>
         </is>
       </c>
     </row>
@@ -877,7 +877,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>56e7134</t>
+          <t>3394712</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>B3 es el HEAD de origin/main al publicar la matriz. Cada fila de 'Matriz Consolidada' tiene su propio SHA en la columna Commit (hipervínculo al diff). Los prompts se leen en rama main: prompts/03_implementacion/.</t>
+          <t>B3 es el HEAD de origin/main al regenerar la matriz. Cada fila de Matriz Consolidada tiene su propio SHA en Commit (F-009 / I-010…I-017 → 3394712). Los prompts se leen en rama main: prompts/03_implementacion/.</t>
         </is>
       </c>
     </row>
@@ -931,7 +931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z9"/>
+  <dimension ref="A1:Z10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="10" customWidth="1" style="14" min="1" max="1"/>
@@ -1136,17 +1136,17 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J2" s="23" t="inlineStr">
+      <c r="J2" s="25" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="K2" s="23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="K2" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L2" s="25" t="inlineStr">
+      <c r="L2" s="26" t="inlineStr">
         <is>
           <t>I-006</t>
         </is>
@@ -1189,19 +1189,19 @@
           <t>src/features/auth/Login.jsx</t>
         </is>
       </c>
-      <c r="U2" s="25" t="inlineStr">
+      <c r="U2" s="26" t="inlineStr">
         <is>
           <t>https://github.com/AxlTech25/Gestion-MPA/blob/5ce7575/src/features/auth/Login.jsx</t>
         </is>
       </c>
-      <c r="V2" s="25" t="inlineStr">
+      <c r="V2" s="26" t="inlineStr">
         <is>
           <t>5ce7575</t>
         </is>
       </c>
       <c r="W2" s="22" t="inlineStr">
         <is>
-          <t>documents/04_testing/plan_pruebas_funcionales.md (casos AUTH)</t>
+          <t>backend/tests/AuthMiddlewareTest.php</t>
         </is>
       </c>
       <c r="X2" s="22" t="inlineStr">
@@ -1216,32 +1216,32 @@
       </c>
       <c r="Z2" s="22" t="inlineStr">
         <is>
-          <t>Origen JWT: 5ce7575 [I-006]. RBAC en servidor: I-009. También AuthMiddleware.php, Jwt.php y AuthContext.jsx.</t>
+          <t>Origen JWT: 5ce7575 [I-006]. RBAC en servidor: I-009. PHPUnit de requireRole. E2E AUTH en plan_pruebas_funcionales.md.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1" s="14">
-      <c r="A3" s="26" t="inlineStr">
+      <c r="A3" s="27" t="inlineStr">
         <is>
           <t>F-002</t>
         </is>
       </c>
-      <c r="B3" s="26" t="inlineStr">
+      <c r="B3" s="27" t="inlineStr">
         <is>
           <t>configuracion</t>
         </is>
       </c>
-      <c r="C3" s="26" t="inlineStr">
-        <is>
-          <t>Áreas y personal (RBAC organizacional)</t>
-        </is>
-      </c>
-      <c r="D3" s="26" t="inlineStr">
+      <c r="C3" s="27" t="inlineStr">
+        <is>
+          <t>Áreas, gerencias y personal (RBAC organizacional)</t>
+        </is>
+      </c>
+      <c r="D3" s="27" t="inlineStr">
         <is>
           <t>Implementación</t>
         </is>
       </c>
-      <c r="E3" s="26" t="inlineStr">
+      <c r="E3" s="27" t="inlineStr">
         <is>
           <t>Presentation (React)</t>
         </is>
@@ -1266,87 +1266,87 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J3" s="23" t="inlineStr">
+      <c r="J3" s="25" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="K3" s="23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="K3" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L3" s="27" t="inlineStr">
+      <c r="L3" s="28" t="inlineStr">
         <is>
           <t>I-005</t>
         </is>
       </c>
-      <c r="M3" s="26" t="inlineStr">
+      <c r="M3" s="27" t="inlineStr">
         <is>
           <t>Few-shot</t>
         </is>
       </c>
-      <c r="N3" s="26" t="inlineStr">
-        <is>
-          <t>v1</t>
-        </is>
-      </c>
-      <c r="O3" s="26" t="n">
-        <v>1</v>
-      </c>
-      <c r="P3" s="26" t="inlineStr">
+      <c r="N3" s="27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="O3" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="P3" s="27" t="inlineStr">
         <is>
           <t>Aprobado</t>
         </is>
       </c>
-      <c r="Q3" s="26" t="inlineStr">
-        <is>
-          <t>CRUD de áreas y usuarios con roles Administrador / Técnico / Practicante</t>
-        </is>
-      </c>
-      <c r="R3" s="26" t="inlineStr">
+      <c r="Q3" s="27" t="inlineStr">
+        <is>
+          <t>CRUD de áreas y gerencias; usuarios con roles Administrador / Técnico / Practicante</t>
+        </is>
+      </c>
+      <c r="R3" s="27" t="inlineStr">
         <is>
           <t>src/features/configuracion/</t>
         </is>
       </c>
-      <c r="S3" s="26" t="inlineStr">
+      <c r="S3" s="27" t="inlineStr">
         <is>
           <t>ConfiguracionPage.jsx</t>
         </is>
       </c>
-      <c r="T3" s="26" t="inlineStr">
+      <c r="T3" s="27" t="inlineStr">
         <is>
           <t>src/features/configuracion/components/ConfiguracionPage.jsx</t>
         </is>
       </c>
-      <c r="U3" s="27" t="inlineStr">
+      <c r="U3" s="28" t="inlineStr">
         <is>
           <t>https://github.com/AxlTech25/Gestion-MPA/blob/4e08b9e/src/features/configuracion/components/ConfiguracionPage.jsx</t>
         </is>
       </c>
-      <c r="V3" s="27" t="inlineStr">
+      <c r="V3" s="28" t="inlineStr">
         <is>
           <t>4e08b9e</t>
         </is>
       </c>
-      <c r="W3" s="26" t="inlineStr">
-        <is>
-          <t>documents/04_testing/plan_pruebas_funcionales.md (casos CFG)</t>
-        </is>
-      </c>
-      <c r="X3" s="26" t="inlineStr">
+      <c r="W3" s="27" t="inlineStr">
+        <is>
+          <t>backend/tests/AreaTest.php</t>
+        </is>
+      </c>
+      <c r="X3" s="27" t="inlineStr">
         <is>
           <t>AxlTech25</t>
         </is>
       </c>
-      <c r="Y3" s="26" t="inlineStr">
+      <c r="Y3" s="27" t="inlineStr">
         <is>
           <t>Desarrollador</t>
         </is>
       </c>
-      <c r="Z3" s="26" t="inlineStr">
-        <is>
-          <t>SHA vigente: 4e08b9e [I-005]. requireRole Administrador: I-009. API: AreaController.php y UsuarioController.php.</t>
+      <c r="Z3" s="27" t="inlineStr">
+        <is>
+          <t>SHA origen: 4e08b9e [I-005]. requireRole: I-009. Gerencias y PUT/DELETE áreas: I-017 (3394712). También UsuarioTest.php.</t>
         </is>
       </c>
     </row>
@@ -1396,7 +1396,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J4" s="28" t="inlineStr">
+      <c r="J4" s="25" t="inlineStr">
         <is>
           <t>Parcial</t>
         </is>
@@ -1406,7 +1406,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="L4" s="25" t="inlineStr">
+      <c r="L4" s="26" t="inlineStr">
         <is>
           <t>I-002</t>
         </is>
@@ -1449,12 +1449,12 @@
           <t>backend/api/v2/controllers/EquipoController.php</t>
         </is>
       </c>
-      <c r="U4" s="25" t="inlineStr">
+      <c r="U4" s="26" t="inlineStr">
         <is>
           <t>https://github.com/AxlTech25/Gestion-MPA/blob/f086a63/backend/api/v2/controllers/EquipoController.php</t>
         </is>
       </c>
-      <c r="V4" s="25" t="inlineStr">
+      <c r="V4" s="26" t="inlineStr">
         <is>
           <t>f086a63</t>
         </is>
@@ -1481,27 +1481,27 @@
       </c>
     </row>
     <row r="5" ht="48" customHeight="1" s="14">
-      <c r="A5" s="26" t="inlineStr">
+      <c r="A5" s="27" t="inlineStr">
         <is>
           <t>F-004</t>
         </is>
       </c>
-      <c r="B5" s="26" t="inlineStr">
+      <c r="B5" s="27" t="inlineStr">
         <is>
           <t>ficha</t>
         </is>
       </c>
-      <c r="C5" s="26" t="inlineStr">
+      <c r="C5" s="27" t="inlineStr">
         <is>
           <t>Ficha técnica y evaluación de hardware/software</t>
         </is>
       </c>
-      <c r="D5" s="26" t="inlineStr">
+      <c r="D5" s="27" t="inlineStr">
         <is>
           <t>Implementación</t>
         </is>
       </c>
-      <c r="E5" s="26" t="inlineStr">
+      <c r="E5" s="27" t="inlineStr">
         <is>
           <t>API (PHP)</t>
         </is>
@@ -1536,75 +1536,75 @@
           <t>No</t>
         </is>
       </c>
-      <c r="L5" s="27" t="inlineStr">
+      <c r="L5" s="28" t="inlineStr">
         <is>
           <t>I-003</t>
         </is>
       </c>
-      <c r="M5" s="26" t="inlineStr">
+      <c r="M5" s="27" t="inlineStr">
         <is>
           <t>Few-shot</t>
         </is>
       </c>
-      <c r="N5" s="26" t="inlineStr">
-        <is>
-          <t>v1</t>
-        </is>
-      </c>
-      <c r="O5" s="26" t="n">
+      <c r="N5" s="27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="O5" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="P5" s="26" t="inlineStr">
+      <c r="P5" s="27" t="inlineStr">
         <is>
           <t>Aprobado</t>
         </is>
       </c>
-      <c r="Q5" s="26" t="inlineStr">
+      <c r="Q5" s="27" t="inlineStr">
         <is>
           <t>Alta/edición de ficha, evaluación y bloque predictivo en UI</t>
         </is>
       </c>
-      <c r="R5" s="26" t="inlineStr">
+      <c r="R5" s="27" t="inlineStr">
         <is>
           <t>backend/api/v2/controllers/</t>
         </is>
       </c>
-      <c r="S5" s="26" t="inlineStr">
+      <c r="S5" s="27" t="inlineStr">
         <is>
           <t>FichaTecnicaController.php</t>
         </is>
       </c>
-      <c r="T5" s="26" t="inlineStr">
+      <c r="T5" s="27" t="inlineStr">
         <is>
           <t>backend/api/v2/controllers/FichaTecnicaController.php</t>
         </is>
       </c>
-      <c r="U5" s="27" t="inlineStr">
+      <c r="U5" s="28" t="inlineStr">
         <is>
           <t>https://github.com/AxlTech25/Gestion-MPA/blob/f086a63/backend/api/v2/controllers/FichaTecnicaController.php</t>
         </is>
       </c>
-      <c r="V5" s="27" t="inlineStr">
+      <c r="V5" s="28" t="inlineStr">
         <is>
           <t>f086a63</t>
         </is>
       </c>
-      <c r="W5" s="26" t="inlineStr">
+      <c r="W5" s="27" t="inlineStr">
         <is>
           <t>documents/04_testing/plan_pruebas_funcionales.md (casos FIC)</t>
         </is>
       </c>
-      <c r="X5" s="26" t="inlineStr">
+      <c r="X5" s="27" t="inlineStr">
         <is>
           <t>AxlTech25</t>
         </is>
       </c>
-      <c r="Y5" s="26" t="inlineStr">
+      <c r="Y5" s="27" t="inlineStr">
         <is>
           <t>Desarrollador</t>
         </is>
       </c>
-      <c r="Z5" s="26" t="inlineStr">
+      <c r="Z5" s="27" t="inlineStr">
         <is>
           <t>SHA vigente: f086a63 [I-003]. Bloque predictivo en ficha: 8b20337 [I-008].</t>
         </is>
@@ -1656,7 +1656,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J6" s="28" t="inlineStr">
+      <c r="J6" s="25" t="inlineStr">
         <is>
           <t>Parcial</t>
         </is>
@@ -1666,7 +1666,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="L6" s="25" t="inlineStr">
+      <c r="L6" s="26" t="inlineStr">
         <is>
           <t>I-003</t>
         </is>
@@ -1709,12 +1709,12 @@
           <t>backend/api/v2/controllers/MantenimientoController.php</t>
         </is>
       </c>
-      <c r="U6" s="25" t="inlineStr">
+      <c r="U6" s="26" t="inlineStr">
         <is>
           <t>https://github.com/AxlTech25/Gestion-MPA/blob/8b20337/backend/api/v2/controllers/MantenimientoController.php</t>
         </is>
       </c>
-      <c r="V6" s="25" t="inlineStr">
+      <c r="V6" s="26" t="inlineStr">
         <is>
           <t>8b20337</t>
         </is>
@@ -1741,27 +1741,27 @@
       </c>
     </row>
     <row r="7" ht="48" customHeight="1" s="14">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="27" t="inlineStr">
         <is>
           <t>F-006</t>
         </is>
       </c>
-      <c r="B7" s="26" t="inlineStr">
+      <c r="B7" s="27" t="inlineStr">
         <is>
           <t>dashboard</t>
         </is>
       </c>
-      <c r="C7" s="26" t="inlineStr">
+      <c r="C7" s="27" t="inlineStr">
         <is>
           <t>Indicadores operativos y consulta de equipos por etiquetas</t>
         </is>
       </c>
-      <c r="D7" s="26" t="inlineStr">
+      <c r="D7" s="27" t="inlineStr">
         <is>
           <t>Implementación</t>
         </is>
       </c>
-      <c r="E7" s="26" t="inlineStr">
+      <c r="E7" s="27" t="inlineStr">
         <is>
           <t>Presentation (React)</t>
         </is>
@@ -1786,7 +1786,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J7" s="28" t="inlineStr">
+      <c r="J7" s="25" t="inlineStr">
         <is>
           <t>Parcial</t>
         </is>
@@ -1796,75 +1796,75 @@
           <t>No</t>
         </is>
       </c>
-      <c r="L7" s="27" t="inlineStr">
+      <c r="L7" s="28" t="inlineStr">
         <is>
           <t>I-006</t>
         </is>
       </c>
-      <c r="M7" s="26" t="inlineStr">
+      <c r="M7" s="27" t="inlineStr">
         <is>
           <t>CoT guiado</t>
         </is>
       </c>
-      <c r="N7" s="26" t="inlineStr">
-        <is>
-          <t>v1</t>
-        </is>
-      </c>
-      <c r="O7" s="26" t="n">
+      <c r="N7" s="27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="O7" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="P7" s="26" t="inlineStr">
+      <c r="P7" s="27" t="inlineStr">
         <is>
           <t>Aprobado</t>
         </is>
       </c>
-      <c r="Q7" s="26" t="inlineStr">
+      <c r="Q7" s="27" t="inlineStr">
         <is>
           <t>Dashboard de métricas, alertas ML y panel de consulta con filtros</t>
         </is>
       </c>
-      <c r="R7" s="26" t="inlineStr">
+      <c r="R7" s="27" t="inlineStr">
         <is>
           <t>src/features/dashboard/</t>
         </is>
       </c>
-      <c r="S7" s="26" t="inlineStr">
+      <c r="S7" s="27" t="inlineStr">
         <is>
           <t>DashboardPage.jsx</t>
         </is>
       </c>
-      <c r="T7" s="26" t="inlineStr">
+      <c r="T7" s="27" t="inlineStr">
         <is>
           <t>src/features/dashboard/components/DashboardPage.jsx</t>
         </is>
       </c>
-      <c r="U7" s="27" t="inlineStr">
+      <c r="U7" s="28" t="inlineStr">
         <is>
           <t>https://github.com/AxlTech25/Gestion-MPA/blob/5ce7575/src/features/dashboard/components/DashboardPage.jsx</t>
         </is>
       </c>
-      <c r="V7" s="27" t="inlineStr">
+      <c r="V7" s="28" t="inlineStr">
         <is>
           <t>5ce7575</t>
         </is>
       </c>
-      <c r="W7" s="26" t="inlineStr">
+      <c r="W7" s="27" t="inlineStr">
         <is>
           <t>backend/tests/DashboardConsultaTest.php</t>
         </is>
       </c>
-      <c r="X7" s="26" t="inlineStr">
+      <c r="X7" s="27" t="inlineStr">
         <is>
           <t>AxlTech25</t>
         </is>
       </c>
-      <c r="Y7" s="26" t="inlineStr">
+      <c r="Y7" s="27" t="inlineStr">
         <is>
           <t>Desarrollador</t>
         </is>
       </c>
-      <c r="Z7" s="26" t="inlineStr">
+      <c r="Z7" s="27" t="inlineStr">
         <is>
           <t>Commit 5ce7575 [I-006] (dashboard de métricas + JWT). Alertas ML: I-007. Consulta tipo_otro: I-008.</t>
         </is>
@@ -1916,7 +1916,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J8" s="28" t="inlineStr">
+      <c r="J8" s="25" t="inlineStr">
         <is>
           <t>Parcial</t>
         </is>
@@ -1926,7 +1926,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="L8" s="25" t="inlineStr">
+      <c r="L8" s="26" t="inlineStr">
         <is>
           <t>I-007</t>
         </is>
@@ -1969,12 +1969,12 @@
           <t>ml/app/main.py</t>
         </is>
       </c>
-      <c r="U8" s="25" t="inlineStr">
+      <c r="U8" s="26" t="inlineStr">
         <is>
           <t>https://github.com/AxlTech25/Gestion-MPA/blob/e9a0965/ml/app/main.py</t>
         </is>
       </c>
-      <c r="V8" s="25" t="inlineStr">
+      <c r="V8" s="26" t="inlineStr">
         <is>
           <t>e9a0965</t>
         </is>
@@ -2001,27 +2001,27 @@
       </c>
     </row>
     <row r="9" ht="48" customHeight="1" s="14">
-      <c r="A9" s="26" t="inlineStr">
+      <c r="A9" s="27" t="inlineStr">
         <is>
           <t>F-008</t>
         </is>
       </c>
-      <c r="B9" s="26" t="inlineStr">
+      <c r="B9" s="27" t="inlineStr">
         <is>
           <t>reportes</t>
         </is>
       </c>
-      <c r="C9" s="26" t="inlineStr">
-        <is>
-          <t>Reportes PDF de ficha técnica y mantenimiento</t>
-        </is>
-      </c>
-      <c r="D9" s="26" t="inlineStr">
+      <c r="C9" s="27" t="inlineStr">
+        <is>
+          <t>Reportes PDF de ficha, mantenimiento y cronograma</t>
+        </is>
+      </c>
+      <c r="D9" s="27" t="inlineStr">
         <is>
           <t>Implementación</t>
         </is>
       </c>
-      <c r="E9" s="26" t="inlineStr">
+      <c r="E9" s="27" t="inlineStr">
         <is>
           <t>API (PHP)</t>
         </is>
@@ -2046,91 +2046,220 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J9" s="23" t="inlineStr">
+      <c r="J9" s="25" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="K9" s="23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="K9" s="23" t="inlineStr">
+      <c r="L9" s="28" t="inlineStr">
+        <is>
+          <t>I-004</t>
+        </is>
+      </c>
+      <c r="M9" s="27" t="inlineStr">
+        <is>
+          <t>Zero-shot + few-shot</t>
+        </is>
+      </c>
+      <c r="N9" s="27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="O9" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="P9" s="27" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="Q9" s="27" t="inlineStr">
+        <is>
+          <t>PDF de ficha, historial de mantenimiento y matriz de cronograma (A4 L–V) con JWT</t>
+        </is>
+      </c>
+      <c r="R9" s="27" t="inlineStr">
+        <is>
+          <t>backend/api/v2/controllers/</t>
+        </is>
+      </c>
+      <c r="S9" s="27" t="inlineStr">
+        <is>
+          <t>ReporteController.php</t>
+        </is>
+      </c>
+      <c r="T9" s="27" t="inlineStr">
+        <is>
+          <t>backend/api/v2/controllers/ReporteController.php</t>
+        </is>
+      </c>
+      <c r="U9" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/AxlTech25/Gestion-MPA/blob/f086a63/backend/api/v2/controllers/ReporteController.php</t>
+        </is>
+      </c>
+      <c r="V9" s="28" t="inlineStr">
+        <is>
+          <t>f086a63</t>
+        </is>
+      </c>
+      <c r="W9" s="27" t="inlineStr">
+        <is>
+          <t>backend/tests/CronogramaTest.php</t>
+        </is>
+      </c>
+      <c r="X9" s="27" t="inlineStr">
+        <is>
+          <t>AxlTech25</t>
+        </is>
+      </c>
+      <c r="Y9" s="27" t="inlineStr">
+        <is>
+          <t>Desarrollador</t>
+        </is>
+      </c>
+      <c r="Z9" s="27" t="inlineStr">
+        <is>
+          <t>SHA origen ficha: f086a63 [I-004]. Descarga JWT: 5ce7575 [I-006]. PDF cronograma (matriz papel A4): I-012…I-016 (3394712).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1" s="14">
+      <c r="A10" s="22" t="inlineStr">
+        <is>
+          <t>F-009</t>
+        </is>
+      </c>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>cronograma</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>Cronograma anual de preventivo (historial, matriz Xn, PDF, gerencias)</t>
+        </is>
+      </c>
+      <c r="D10" s="22" t="inlineStr">
+        <is>
+          <t>Implementación</t>
+        </is>
+      </c>
+      <c r="E10" s="22" t="inlineStr">
+        <is>
+          <t>Presentation (React)</t>
+        </is>
+      </c>
+      <c r="F10" s="23" t="inlineStr">
+        <is>
+          <t>Alto (integración/validación)</t>
+        </is>
+      </c>
+      <c r="G10" s="24" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H10" s="23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L9" s="27" t="inlineStr">
-        <is>
-          <t>I-004</t>
-        </is>
-      </c>
-      <c r="M9" s="26" t="inlineStr">
-        <is>
-          <t>Zero-shot + few-shot</t>
-        </is>
-      </c>
-      <c r="N9" s="26" t="inlineStr">
-        <is>
-          <t>v1</t>
-        </is>
-      </c>
-      <c r="O9" s="26" t="n">
-        <v>1</v>
-      </c>
-      <c r="P9" s="26" t="inlineStr">
+      <c r="I10" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J10" s="25" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="K10" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L10" s="26" t="inlineStr">
+        <is>
+          <t>I-010</t>
+        </is>
+      </c>
+      <c r="M10" s="22" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="N10" s="22" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="O10" s="22" t="n">
+        <v>7</v>
+      </c>
+      <c r="P10" s="22" t="inlineStr">
         <is>
           <t>Aprobado</t>
         </is>
       </c>
-      <c r="Q9" s="26" t="inlineStr">
-        <is>
-          <t>PDF de ficha de equipo e historial/detalle de mantenimiento con JWT en descarga</t>
-        </is>
-      </c>
-      <c r="R9" s="26" t="inlineStr">
-        <is>
-          <t>backend/api/v2/controllers/</t>
-        </is>
-      </c>
-      <c r="S9" s="26" t="inlineStr">
-        <is>
-          <t>ReporteController.php</t>
-        </is>
-      </c>
-      <c r="T9" s="26" t="inlineStr">
-        <is>
-          <t>backend/api/v2/controllers/ReporteController.php</t>
-        </is>
-      </c>
-      <c r="U9" s="27" t="inlineStr">
-        <is>
-          <t>https://github.com/AxlTech25/Gestion-MPA/blob/f086a63/backend/api/v2/controllers/ReporteController.php</t>
-        </is>
-      </c>
-      <c r="V9" s="27" t="inlineStr">
-        <is>
-          <t>f086a63</t>
-        </is>
-      </c>
-      <c r="W9" s="26" t="inlineStr">
-        <is>
-          <t>documents/04_testing/plan_pruebas_funcionales.md (casos RPT)</t>
-        </is>
-      </c>
-      <c r="X9" s="26" t="inlineStr">
+      <c r="Q10" s="22" t="inlineStr">
+        <is>
+          <t>Historial de planes, matriz área×día×cantidad, personal, PDF A4 y bandas de gerencia</t>
+        </is>
+      </c>
+      <c r="R10" s="22" t="inlineStr">
+        <is>
+          <t>src/features/cronograma/</t>
+        </is>
+      </c>
+      <c r="S10" s="22" t="inlineStr">
+        <is>
+          <t>CronogramaMatrizPage.jsx</t>
+        </is>
+      </c>
+      <c r="T10" s="22" t="inlineStr">
+        <is>
+          <t>src/features/cronograma/components/CronogramaMatrizPage.jsx</t>
+        </is>
+      </c>
+      <c r="U10" s="26" t="inlineStr">
+        <is>
+          <t>https://github.com/AxlTech25/Gestion-MPA/blob/3394712/src/features/cronograma/components/CronogramaMatrizPage.jsx</t>
+        </is>
+      </c>
+      <c r="V10" s="26" t="inlineStr">
+        <is>
+          <t>3394712</t>
+        </is>
+      </c>
+      <c r="W10" s="22" t="inlineStr">
+        <is>
+          <t>backend/tests/CronogramaTest.php</t>
+        </is>
+      </c>
+      <c r="X10" s="22" t="inlineStr">
         <is>
           <t>AxlTech25</t>
         </is>
       </c>
-      <c r="Y9" s="26" t="inlineStr">
+      <c r="Y10" s="22" t="inlineStr">
         <is>
           <t>Desarrollador</t>
         </is>
       </c>
-      <c r="Z9" s="26" t="inlineStr">
-        <is>
-          <t>SHA vigente: f086a63 [I-004]. Descarga con JWT (blob): 5ce7575 [I-006].</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="29" customHeight="1" s="14"/>
+      <c r="Z10" s="22" t="inlineStr">
+        <is>
+          <t>Incremento 8 cerrado 2026-09-17 (0.10.0–0.10.7). Origen I-010; parches I-011…I-017. SHA: 3394712. También cronogramaUtils.test.js. API: CronogramaController.php.</t>
+        </is>
+      </c>
+    </row>
     <row r="11" ht="29" customHeight="1" s="14"/>
     <row r="12" ht="29" customHeight="1" s="14"/>
     <row r="13" ht="29" customHeight="1" s="14"/>
@@ -2141,7 +2270,7 @@
     <row r="18" ht="29" customHeight="1" s="14"/>
     <row r="20" ht="29" customHeight="1" s="14"/>
   </sheetData>
-  <autoFilter ref="A1:Z9"/>
+  <autoFilter ref="A1:Z10"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U2" r:id="rId2"/>
@@ -2167,6 +2296,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U9" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V9" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U10" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V10" r:id="rId27"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2178,7 +2310,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="12" customWidth="1" style="14" min="1" max="1"/>
@@ -2250,7 +2382,7 @@
       </c>
     </row>
     <row r="2" ht="90" customHeight="1" s="14">
-      <c r="A2" s="25" t="inlineStr">
+      <c r="A2" s="26" t="inlineStr">
         <is>
           <t>I-006</t>
         </is>
@@ -2298,69 +2430,69 @@
           <t>Login JWT funcional (AuthContext, PrivateRoute, middleware)</t>
         </is>
       </c>
-      <c r="K2" s="25" t="inlineStr">
+      <c r="K2" s="26" t="inlineStr">
         <is>
           <t>5ce7575</t>
         </is>
       </c>
     </row>
     <row r="3" ht="90" customHeight="1" s="14">
-      <c r="A3" s="27" t="inlineStr">
+      <c r="A3" s="28" t="inlineStr">
         <is>
           <t>I-005</t>
         </is>
       </c>
-      <c r="B3" s="26" t="inlineStr">
+      <c r="B3" s="27" t="inlineStr">
         <is>
           <t>F-002</t>
         </is>
       </c>
-      <c r="C3" s="26" t="inlineStr">
+      <c r="C3" s="27" t="inlineStr">
         <is>
           <t>Actúa como desarrollador senior PHP/React. Contexto: áreas y responsables no deben estar hardcodeados en EquipoForm; tablas v2_areas y v2_usuarios existen; ruta /v2/configuracion; roles Administrador, Tecnico, Practicante. Objetivo: CRUD de áreas y alta/listado de personal. Tarea: modelos PDO; password_hash BCRYPT; rutas /areas y /usuarios; ConfiguracionPage (pestañas); EquipoForm consume áreas desde API. Restricciones: no MD5; no requireRole en este incremento (deuda → I-009). Criterios: crear un área y verla en EquipoForm; usuario con hash en BD.</t>
         </is>
       </c>
-      <c r="D3" s="26" t="inlineStr">
+      <c r="D3" s="27" t="inlineStr">
         <is>
           <t>Few-shot</t>
         </is>
       </c>
-      <c r="E3" s="26" t="inlineStr">
-        <is>
-          <t>v1</t>
-        </is>
-      </c>
-      <c r="F3" s="26" t="n">
+      <c r="E3" s="27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F3" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="G3" s="26" t="inlineStr">
+      <c r="G3" s="27" t="inlineStr">
         <is>
           <t>La API de usuarios quedó solo autenticada. I-009 añade requireRole Administrador.</t>
         </is>
       </c>
-      <c r="H3" s="26" t="inlineStr">
-        <is>
-          <t>v1</t>
-        </is>
-      </c>
-      <c r="I3" s="26" t="inlineStr">
+      <c r="H3" s="27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I3" s="27" t="inlineStr">
         <is>
           <t>Aprobado</t>
         </is>
       </c>
-      <c r="J3" s="26" t="inlineStr">
+      <c r="J3" s="27" t="inlineStr">
         <is>
           <t>Áreas y personal funcionales; EquipoForm dinámico</t>
         </is>
       </c>
-      <c r="K3" s="27" t="inlineStr">
+      <c r="K3" s="28" t="inlineStr">
         <is>
           <t>4e08b9e</t>
         </is>
       </c>
     </row>
     <row r="4" ht="90" customHeight="1" s="14">
-      <c r="A4" s="25" t="inlineStr">
+      <c r="A4" s="26" t="inlineStr">
         <is>
           <t>I-002</t>
         </is>
@@ -2408,69 +2540,69 @@
           <t>CRUD de equipos con código de 12 dígitos y RAM numérica</t>
         </is>
       </c>
-      <c r="K4" s="25" t="inlineStr">
+      <c r="K4" s="26" t="inlineStr">
         <is>
           <t>f086a63</t>
         </is>
       </c>
     </row>
     <row r="5" ht="90" customHeight="1" s="14">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="28" t="inlineStr">
         <is>
           <t>I-003</t>
         </is>
       </c>
-      <c r="B5" s="26" t="inlineStr">
+      <c r="B5" s="27" t="inlineStr">
         <is>
           <t>F-004</t>
         </is>
       </c>
-      <c r="C5" s="26" t="inlineStr">
+      <c r="C5" s="27" t="inlineStr">
         <is>
           <t>Actúa como desarrollador senior PHP/React; replica el patrón I-002. Contexto: equipos ya se listan; hace falta consultar/editar ficha técnica del equipo. Tarea: modelo/controlador/ruta de fichas; GET por id y por código patrimonial; acceso desde inventario (modal o /v2/ficha-tecnica). Restricciones: no PDF (I-004); no bloque ML (I-008). Criterios: GET ficha existente o vacío controlado (no 500).</t>
         </is>
       </c>
-      <c r="D5" s="26" t="inlineStr">
+      <c r="D5" s="27" t="inlineStr">
         <is>
           <t>Few-shot</t>
         </is>
       </c>
-      <c r="E5" s="26" t="inlineStr">
-        <is>
-          <t>v1</t>
-        </is>
-      </c>
-      <c r="F5" s="26" t="n">
+      <c r="E5" s="27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F5" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="26" t="inlineStr">
+      <c r="G5" s="27" t="inlineStr">
         <is>
           <t>N/A — evaluación predictiva en ficha es I-008.</t>
         </is>
       </c>
-      <c r="H5" s="26" t="inlineStr">
-        <is>
-          <t>v1</t>
-        </is>
-      </c>
-      <c r="I5" s="26" t="inlineStr">
+      <c r="H5" s="27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I5" s="27" t="inlineStr">
         <is>
           <t>Aprobado</t>
         </is>
       </c>
-      <c r="J5" s="26" t="inlineStr">
+      <c r="J5" s="27" t="inlineStr">
         <is>
           <t>API y UI de ficha técnica por id o código</t>
         </is>
       </c>
-      <c r="K5" s="27" t="inlineStr">
+      <c r="K5" s="28" t="inlineStr">
         <is>
           <t>f086a63</t>
         </is>
       </c>
     </row>
     <row r="6" ht="90" customHeight="1" s="14">
-      <c r="A6" s="25" t="inlineStr">
+      <c r="A6" s="26" t="inlineStr">
         <is>
           <t>I-003</t>
         </is>
@@ -2518,69 +2650,69 @@
           <t>Timeline y alta estructurada de mantenimientos</t>
         </is>
       </c>
-      <c r="K6" s="25" t="inlineStr">
+      <c r="K6" s="26" t="inlineStr">
         <is>
           <t>8b20337</t>
         </is>
       </c>
     </row>
     <row r="7" ht="90" customHeight="1" s="14">
-      <c r="A7" s="27" t="inlineStr">
+      <c r="A7" s="28" t="inlineStr">
         <is>
           <t>I-006</t>
         </is>
       </c>
-      <c r="B7" s="26" t="inlineStr">
+      <c r="B7" s="27" t="inlineStr">
         <is>
           <t>F-006</t>
         </is>
       </c>
-      <c r="C7" s="26" t="inlineStr">
+      <c r="C7" s="27" t="inlineStr">
         <is>
           <t>Actúa como desarrollador senior PHP/React (mismo incremento 0.6.0 que F-001). Objetivo: métricas operativas en GET /api/v2/dashboard y UI DashboardPage (conteos, no ML). Tarea: DashboardController + DashboardPage; no badges de riesgo (I-007); no panel de consulta por etiquetas (I-008). Restricciones: no llamar a :8000. Criterios: dashboard muestra conteos persistidos tras login.</t>
         </is>
       </c>
-      <c r="D7" s="26" t="inlineStr">
+      <c r="D7" s="27" t="inlineStr">
         <is>
           <t>CoT guiado</t>
         </is>
       </c>
-      <c r="E7" s="26" t="inlineStr">
-        <is>
-          <t>v1</t>
-        </is>
-      </c>
-      <c r="F7" s="26" t="n">
+      <c r="E7" s="27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F7" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="26" t="inlineStr">
+      <c r="G7" s="27" t="inlineStr">
         <is>
           <t>N/A — consulta tipo_otro es I-008; alertas ML son I-007.</t>
         </is>
       </c>
-      <c r="H7" s="26" t="inlineStr">
-        <is>
-          <t>v1</t>
-        </is>
-      </c>
-      <c r="I7" s="26" t="inlineStr">
+      <c r="H7" s="27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I7" s="27" t="inlineStr">
         <is>
           <t>Aprobado</t>
         </is>
       </c>
-      <c r="J7" s="26" t="inlineStr">
+      <c r="J7" s="27" t="inlineStr">
         <is>
           <t>Dashboard de métricas operativas funcional</t>
         </is>
       </c>
-      <c r="K7" s="27" t="inlineStr">
+      <c r="K7" s="28" t="inlineStr">
         <is>
           <t>5ce7575</t>
         </is>
       </c>
     </row>
     <row r="8" ht="90" customHeight="1" s="14">
-      <c r="A8" s="25" t="inlineStr">
+      <c r="A8" s="26" t="inlineStr">
         <is>
           <t>I-007</t>
         </is>
@@ -2628,69 +2760,69 @@
           <t>FastAPI + proxy PHP + badges; degradación controlada</t>
         </is>
       </c>
-      <c r="K8" s="25" t="inlineStr">
+      <c r="K8" s="26" t="inlineStr">
         <is>
           <t>e9a0965</t>
         </is>
       </c>
     </row>
     <row r="9" ht="90" customHeight="1" s="14">
-      <c r="A9" s="27" t="inlineStr">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>I-004</t>
         </is>
       </c>
-      <c r="B9" s="26" t="inlineStr">
+      <c r="B9" s="27" t="inlineStr">
         <is>
           <t>F-008</t>
         </is>
       </c>
-      <c r="C9" s="26" t="inlineStr">
+      <c r="C9" s="27" t="inlineStr">
         <is>
           <t>Actúa como desarrollador senior PHP (dompdf) y React. Contexto: inventario y ficha ya existen. Objetivo: GET /api/v2/reportes/equipo/{id} genera PDF; InventarioPage filtra en cliente y ofrece descargar ficha. Tarea: Composer dompdf; ReporteController HTML→PDF; botón en la fila. Restricciones: PDF binario, no base64; no reportes de mantenimiento en este incremento. Criterios: PDF muestra código patrimonial; filtro de texto reduce filas.</t>
         </is>
       </c>
-      <c r="D9" s="26" t="inlineStr">
+      <c r="D9" s="27" t="inlineStr">
         <is>
           <t>Zero-shot + few-shot</t>
         </is>
       </c>
-      <c r="E9" s="26" t="inlineStr">
-        <is>
-          <t>v1</t>
-        </is>
-      </c>
-      <c r="F9" s="26" t="n">
+      <c r="E9" s="27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="26" t="inlineStr">
+      <c r="G9" s="27" t="inlineStr">
         <is>
           <t>window.open sin token; I-006 cambia la descarga a blob + Authorization.</t>
         </is>
       </c>
-      <c r="H9" s="26" t="inlineStr">
-        <is>
-          <t>v1</t>
-        </is>
-      </c>
-      <c r="I9" s="26" t="inlineStr">
+      <c r="H9" s="27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I9" s="27" t="inlineStr">
         <is>
           <t>Aprobado</t>
         </is>
       </c>
-      <c r="J9" s="26" t="inlineStr">
+      <c r="J9" s="27" t="inlineStr">
         <is>
           <t>PDF de ficha y filtros de inventario funcionales</t>
         </is>
       </c>
-      <c r="K9" s="27" t="inlineStr">
+      <c r="K9" s="28" t="inlineStr">
         <is>
           <t>f086a63</t>
         </is>
       </c>
     </row>
     <row r="10" ht="90" customHeight="1" s="14">
-      <c r="A10" s="25" t="inlineStr">
+      <c r="A10" s="26" t="inlineStr">
         <is>
           <t>I-008</t>
         </is>
@@ -2738,64 +2870,504 @@
           <t>Telemetría, sync, ficha predictiva y consulta de equipos</t>
         </is>
       </c>
-      <c r="K10" s="25" t="inlineStr">
+      <c r="K10" s="26" t="inlineStr">
         <is>
           <t>8b20337</t>
         </is>
       </c>
     </row>
     <row r="11" ht="90" customHeight="1" s="14">
-      <c r="A11" s="27" t="inlineStr">
+      <c r="A11" s="28" t="inlineStr">
         <is>
           <t>I-009</t>
         </is>
       </c>
-      <c r="B11" s="26" t="inlineStr">
+      <c r="B11" s="27" t="inlineStr">
         <is>
           <t>F-001, F-002, F-003</t>
         </is>
       </c>
-      <c r="C11" s="26" t="inlineStr">
+      <c r="C11" s="27" t="inlineStr">
         <is>
           <t>Actúa como desarrollador senior de API PHP y React. Contexto: 0.9.1; JWT existe; un Técnico puede mutar /usuarios; plantilla Excel desalinea numero_serie/area por falta de color. Objetivo: requireRole Administrador en escritura de usuarios; no autoeliminación ni borrar el último admin; RoleRoute en Configuración; fila ejemplo Excel alineada. Criterios: Técnico en POST /usuarios → 403.</t>
         </is>
       </c>
-      <c r="D11" s="26" t="inlineStr">
+      <c r="D11" s="27" t="inlineStr">
         <is>
           <t>CoT guiado</t>
         </is>
       </c>
-      <c r="E11" s="26" t="inlineStr">
-        <is>
-          <t>v1</t>
-        </is>
-      </c>
-      <c r="F11" s="26" t="n">
+      <c r="E11" s="27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F11" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="G11" s="26" t="inlineStr">
+      <c r="G11" s="27" t="inlineStr">
         <is>
           <t>I-005 no puso autorización en servidor (deuda de RBAC).</t>
         </is>
       </c>
-      <c r="H11" s="26" t="inlineStr">
-        <is>
-          <t>v1</t>
-        </is>
-      </c>
-      <c r="I11" s="26" t="inlineStr">
+      <c r="H11" s="27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I11" s="27" t="inlineStr">
         <is>
           <t>Aprobado</t>
         </is>
       </c>
-      <c r="J11" s="26" t="inlineStr">
+      <c r="J11" s="27" t="inlineStr">
         <is>
           <t>requireRole en /usuarios y plantilla Excel alineada</t>
         </is>
       </c>
-      <c r="K11" s="27" t="inlineStr">
+      <c r="K11" s="28" t="inlineStr">
         <is>
           <t>8b20337</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="90" customHeight="1" s="14">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>I-010</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>F-009</t>
+        </is>
+      </c>
+      <c r="C12" s="22" t="inlineStr">
+        <is>
+          <t>Actúa como desarrollador senior PHP 8 / React 19. Contexto: 0.9.1; R-006 y D-007; ADR-003 (v2_cronogramas / v2_cronograma_celdas); no usar v2_cronograma_mantenimiento. Objetivo: historial, alta de documento, matriz área×día×turno, cobertura y PDF. Tarea: SQL+migrate; modelo; controller; GET /reportes/cronograma/{id}; feature cronograma; Navbar; PHPUnit/Vitest. Restricciones: no ML; no dual-write; Practicante GET sí / POST 403. Criterios: dos planes el mismo año; clic crea/libera celda; PDF autenticado.</t>
+        </is>
+      </c>
+      <c r="D12" s="22" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="E12" s="22" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F12" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="22" t="inlineStr">
+        <is>
+          <t>N/A en origen. Totales, PDF papel, Xn, A4, gerencias = I-011…I-017.</t>
+        </is>
+      </c>
+      <c r="H12" s="22" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I12" s="22" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="J12" s="22" t="inlineStr">
+        <is>
+          <t>Historial, matriz y PDF autenticado (0.10.0)</t>
+        </is>
+      </c>
+      <c r="K12" s="26" t="inlineStr">
+        <is>
+          <t>3394712</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="90" customHeight="1" s="14">
+      <c r="A13" s="28" t="inlineStr">
+        <is>
+          <t>I-011</t>
+        </is>
+      </c>
+      <c r="B13" s="27" t="inlineStr">
+        <is>
+          <t>F-009</t>
+        </is>
+      </c>
+      <c r="C13" s="27" t="inlineStr">
+        <is>
+          <t>Actúa como desarrollador senior PHP 8 / React 19. Contexto: 0.10.0. Faltan subtotal/total; hay que programar hora de cada equipo; Imprimir PDF abre pestaña en blanco. Objetivo: parche 0.10.1. El asiento sigue área+fecha+turno (ADR-003). Tarea: columna Tot y pie Subtotal/Total; v2_cronograma_horarios + modal PUT; downloadPdf con attachment y Content-Type PDF. Criterios: pie de totales; modal horas; PDF descarga archivo.</t>
+        </is>
+      </c>
+      <c r="D13" s="27" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="E13" s="27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F13" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="27" t="inlineStr">
+        <is>
+          <t>I-010 no tenía totales ni horas por equipo; downloadPdf sin attachment.</t>
+        </is>
+      </c>
+      <c r="H13" s="27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I13" s="27" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="J13" s="27" t="inlineStr">
+        <is>
+          <t>Totales, horarios por equipo e impresión con download</t>
+        </is>
+      </c>
+      <c r="K13" s="28" t="inlineStr">
+        <is>
+          <t>3394712</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="90" customHeight="1" s="14">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>I-012</t>
+        </is>
+      </c>
+      <c r="B14" s="22" t="inlineStr">
+        <is>
+          <t>F-008, F-009</t>
+        </is>
+      </c>
+      <c r="C14" s="22" t="inlineStr">
+        <is>
+          <t>Actúa como desarrollador senior PHP 8 / Dompdf. Contexto: el PDF era un listado; el papel 2024 es una matriz N°/área/PC/laptop/impresora × meses y días con marcas X1/X2. Objetivo: GET /reportes/cronograma/{id} imprime esa grilla. Tarea: A3 apaisado; rango de meses con marca; un día = una columna; última hoja leyenda y nota. No cambiar el asiento. Criterios: el PDF se parece al papel; las X coinciden con la UI.</t>
+        </is>
+      </c>
+      <c r="D14" s="22" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="E14" s="22" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F14" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="22" t="inlineStr">
+        <is>
+          <t>I-011 imprimía listado, no la grilla del papel.</t>
+        </is>
+      </c>
+      <c r="H14" s="22" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I14" s="22" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="J14" s="22" t="inlineStr">
+        <is>
+          <t>PDF tipo matriz (papel 2024)</t>
+        </is>
+      </c>
+      <c r="K14" s="26" t="inlineStr">
+        <is>
+          <t>3394712</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="90" customHeight="1" s="14">
+      <c r="A15" s="28" t="inlineStr">
+        <is>
+          <t>I-013</t>
+        </is>
+      </c>
+      <c r="B15" s="27" t="inlineStr">
+        <is>
+          <t>F-009</t>
+        </is>
+      </c>
+      <c r="C15" s="27" t="inlineStr">
+        <is>
+          <t>Actúa como desarrollador senior PHP 8 / React 19. Contexto: el recuadro HORA PROGRAMADA del papel son las personas que hacen el preventivo, no los bienes del área. Objetivo: recuadro editable en matriz y PDF. Tarea: v2_cronograma_personal; PUT /cronogramas/{id}/personal; quitar del PDF la tabla grande de horas por CPU. Criterios: se edita el nombre y se ve igual en el PDF.</t>
+        </is>
+      </c>
+      <c r="D15" s="27" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="E15" s="27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F15" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="27" t="inlineStr">
+        <is>
+          <t>I-012 listaba PCs del inventario en HORA PROGRAMADA; el papel lista personas.</t>
+        </is>
+      </c>
+      <c r="H15" s="27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I15" s="27" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="J15" s="27" t="inlineStr">
+        <is>
+          <t>Personal del preventivo en HORA PROGRAMADA</t>
+        </is>
+      </c>
+      <c r="K15" s="28" t="inlineStr">
+        <is>
+          <t>3394712</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="90" customHeight="1" s="14">
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>I-014</t>
+        </is>
+      </c>
+      <c r="B16" s="22" t="inlineStr">
+        <is>
+          <t>F-009</t>
+        </is>
+      </c>
+      <c r="C16" s="22" t="inlineStr">
+        <is>
+          <t>Actúa como desarrollador senior PHP 8 / React 19. Contexto: X1/X2 no son mañana/tarde: son cuántos PC/laptop se atienden ese día. Objetivo: asiento = cronograma + área + fecha + cantidad; una columna por día. Tarea: SQL cantidad + UNIQUE(área,fecha); POST {cantidad}; selector X1…Xn; cobertura = suma(cantidad) vs PC+laptop. Restricciones: no 10 columnas; no auto-fill; impresoras no entran en Xn.</t>
+        </is>
+      </c>
+      <c r="D16" s="22" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="E16" s="22" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F16" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="22" t="inlineStr">
+        <is>
+          <t>I-010 modeló X1/X2 como turnos; el papel usa cantidad por día.</t>
+        </is>
+      </c>
+      <c r="H16" s="22" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I16" s="22" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="J16" s="22" t="inlineStr">
+        <is>
+          <t>Xn = cantidad por día (no turnos)</t>
+        </is>
+      </c>
+      <c r="K16" s="26" t="inlineStr">
+        <is>
+          <t>3394712</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="90" customHeight="1" s="14">
+      <c r="A17" s="28" t="inlineStr">
+        <is>
+          <t>I-015</t>
+        </is>
+      </c>
+      <c r="B17" s="27" t="inlineStr">
+        <is>
+          <t>F-009</t>
+        </is>
+      </c>
+      <c r="C17" s="27" t="inlineStr">
+        <is>
+          <t>Actúa como desarrollador senior PHP 8 / React 19 / Dompdf. Contexto: PDF A3 4 meses con sábados/domingos; hace falta A4, L–V, 2 meses/hoja, año del documento y poder borrar un plan. Objetivo: PDF A4 apaisado laborable; DELETE /cronogramas/{id} CASCADE; matriz UI sin fines de semana. Restricciones: no auto-fill; Practicante no elimina; conservar N°/área/conteos.</t>
+        </is>
+      </c>
+      <c r="D17" s="27" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="E17" s="27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F17" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="27" t="inlineStr">
+        <is>
+          <t>I-012 era A3 calendario completo; el responsable pidió A4 laborable y baja.</t>
+        </is>
+      </c>
+      <c r="H17" s="27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I17" s="27" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="J17" s="27" t="inlineStr">
+        <is>
+          <t>PDF A4 L–V 2 meses/hoja y DELETE del plan</t>
+        </is>
+      </c>
+      <c r="K17" s="28" t="inlineStr">
+        <is>
+          <t>3394712</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="90" customHeight="1" s="14">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>I-016</t>
+        </is>
+      </c>
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>F-008, F-009</t>
+        </is>
+      </c>
+      <c r="C18" s="22" t="inlineStr">
+        <is>
+          <t>Actúa como desarrollador senior PHP 8 / Dompdf. Contexto: el PDF A4 aplastaba ÁREA (colspan calendario vs L–V); N° enorme; PC/LAP/IMP acrónimos; dos tablas desalineadas; HORA PROGRAMADA sin reja. Objetivo: una sola tabla; textos sin distorsión; pie N°/EQUIPO/HORARIO con borde. Criterios: áreas se leen; PC/LAPTOP/IMPRESORA completos; filas Xn alineadas.</t>
+        </is>
+      </c>
+      <c r="D18" s="22" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="E18" s="22" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F18" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="22" t="inlineStr">
+        <is>
+          <t>I-015 encajaba mal colspan y el pie no tenía borde.</t>
+        </is>
+      </c>
+      <c r="H18" s="22" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I18" s="22" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="J18" s="22" t="inlineStr">
+        <is>
+          <t>PDF encajado; HORA PROGRAMADA con borde</t>
+        </is>
+      </c>
+      <c r="K18" s="26" t="inlineStr">
+        <is>
+          <t>3394712</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="90" customHeight="1" s="14">
+      <c r="A19" s="28" t="inlineStr">
+        <is>
+          <t>I-017</t>
+        </is>
+      </c>
+      <c r="B19" s="27" t="inlineStr">
+        <is>
+          <t>F-002, F-009</t>
+        </is>
+      </c>
+      <c r="C19" s="27" t="inlineStr">
+        <is>
+          <t>Actúa como desarrollador senior PHP 8 / React 19. Contexto: el papel agrupa áreas bajo filas de gerencia; v2_areas solo tenía alta. Objetivo: catálogo v2_gerencias; área.gerencia_id; CRUD de área (Admin); matriz y PDF con fila banda. Restricciones: no auto-fill; SIGA/SAF son áreas, no gerencias; no borrar área con equipos (409); no etiqueta libre. Criterios: asignar gerencia; 409 si hay equipos; bandas en cronograma/PDF.</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="E19" s="27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F19" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="27" t="inlineStr">
+        <is>
+          <t>Cierre del Incremento 8: gerencias del papel y CRUD de áreas pendiente desde I-005.</t>
+        </is>
+      </c>
+      <c r="H19" s="27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I19" s="27" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="J19" s="27" t="inlineStr">
+        <is>
+          <t>Gerencias, CRUD de áreas y bandas en cronograma (0.10.7)</t>
+        </is>
+      </c>
+      <c r="K19" s="28" t="inlineStr">
+        <is>
+          <t>3394712</t>
         </is>
       </c>
     </row>
@@ -2821,6 +3393,22 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3052,7 +3640,7 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Identificador del prompt vigente (I-002…I-009). Una fila por función F-001…F-008 en Prompts Detallados. Hipervínculo al markdown en GitHub (prompts/).</t>
+          <t>Identificador del prompt vigente (I-002…I-017). Una fila por función F-001…F-009 en Prompts Detallados, más refinamientos. Hipervínculo al markdown en GitHub (prompts/).</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">

</xml_diff>